<commit_message>
Excel files for pulm
</commit_message>
<xml_diff>
--- a/BVSimulationFiles/53.xlsx
+++ b/BVSimulationFiles/53.xlsx
@@ -1,38 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cbnor\Documents\Full Body Flow Model Project\BVSimulationFiles\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BB7EEC9-82AE-4C71-9485-ABEDDE0B3527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="1103" yWindow="1103" windowWidth="16200" windowHeight="9307" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -51,21 +47,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -353,200 +408,204 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:U3"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.45">
-      <c r="B1">
+    <row r="1">
+      <c r="B1" t="n">
         <v>0</v>
       </c>
-      <c r="C1">
-        <v>1.568947368421053E-3</v>
-      </c>
-      <c r="D1">
-        <v>3.1378947368421051E-3</v>
-      </c>
-      <c r="E1">
-        <v>4.7068421052631577E-3</v>
-      </c>
-      <c r="F1">
-        <v>6.2757894736842103E-3</v>
-      </c>
-      <c r="G1">
-        <v>7.844736842105262E-3</v>
-      </c>
-      <c r="H1">
-        <v>9.4136842105263154E-3</v>
-      </c>
-      <c r="I1">
-        <v>1.0982631578947371E-2</v>
-      </c>
-      <c r="J1">
-        <v>1.2551578947368421E-2</v>
-      </c>
-      <c r="K1">
-        <v>1.4120526315789471E-2</v>
-      </c>
-      <c r="L1">
-        <v>1.568947368421052E-2</v>
-      </c>
-      <c r="M1">
-        <v>1.7258421052631579E-2</v>
-      </c>
-      <c r="N1">
-        <v>1.8827368421052631E-2</v>
-      </c>
-      <c r="O1">
-        <v>2.0396315789473679E-2</v>
-      </c>
-      <c r="P1">
-        <v>2.1965263157894741E-2</v>
-      </c>
-      <c r="Q1">
-        <v>2.3534210526315789E-2</v>
-      </c>
-      <c r="R1">
-        <v>2.5103157894736841E-2</v>
-      </c>
-      <c r="S1">
-        <v>2.66721052631579E-2</v>
-      </c>
-      <c r="T1">
-        <v>2.8241052631578941E-2</v>
-      </c>
-      <c r="U1">
-        <v>2.981E-2</v>
+      <c r="C1" t="n">
+        <v>0.001568947368421053</v>
+      </c>
+      <c r="D1" t="n">
+        <v>0.003137894736842105</v>
+      </c>
+      <c r="E1" t="n">
+        <v>0.004706842105263158</v>
+      </c>
+      <c r="F1" t="n">
+        <v>0.00627578947368421</v>
+      </c>
+      <c r="G1" t="n">
+        <v>0.007844736842105262</v>
+      </c>
+      <c r="H1" t="n">
+        <v>0.009413684210526315</v>
+      </c>
+      <c r="I1" t="n">
+        <v>0.01098263157894737</v>
+      </c>
+      <c r="J1" t="n">
+        <v>0.01255157894736842</v>
+      </c>
+      <c r="K1" t="n">
+        <v>0.01412052631578947</v>
+      </c>
+      <c r="L1" t="n">
+        <v>0.01568947368421052</v>
+      </c>
+      <c r="M1" t="n">
+        <v>0.01725842105263158</v>
+      </c>
+      <c r="N1" t="n">
+        <v>0.01882736842105263</v>
+      </c>
+      <c r="O1" t="n">
+        <v>0.02039631578947368</v>
+      </c>
+      <c r="P1" t="n">
+        <v>0.02196526315789474</v>
+      </c>
+      <c r="Q1" t="n">
+        <v>0.02353421052631579</v>
+      </c>
+      <c r="R1" t="n">
+        <v>0.02510315789473684</v>
+      </c>
+      <c r="S1" t="n">
+        <v>0.0266721052631579</v>
+      </c>
+      <c r="T1" t="n">
+        <v>0.02824105263157894</v>
+      </c>
+      <c r="U1" t="n">
+        <v>0.02981</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.45">
-      <c r="A2">
+    <row r="2">
+      <c r="A2" t="n">
         <v>0</v>
       </c>
-      <c r="B2">
-        <v>8.8998035363457764E-3</v>
-      </c>
-      <c r="C2">
-        <v>8.9380622479578124E-3</v>
-      </c>
-      <c r="D2">
-        <v>8.9763209595698484E-3</v>
-      </c>
-      <c r="E2">
-        <v>9.0145796711818844E-3</v>
-      </c>
-      <c r="F2">
-        <v>9.0528383827939204E-3</v>
-      </c>
-      <c r="G2">
-        <v>9.0910970944059546E-3</v>
-      </c>
-      <c r="H2">
-        <v>9.1293558060179907E-3</v>
-      </c>
-      <c r="I2">
-        <v>9.1676145176300284E-3</v>
-      </c>
-      <c r="J2">
-        <v>9.2058732292420644E-3</v>
-      </c>
-      <c r="K2">
-        <v>9.2441319408541004E-3</v>
-      </c>
-      <c r="L2">
-        <v>9.2823906524661347E-3</v>
-      </c>
-      <c r="M2">
-        <v>9.3206493640781724E-3</v>
-      </c>
-      <c r="N2">
-        <v>9.3589080756902084E-3</v>
-      </c>
-      <c r="O2">
-        <v>9.3971667873022427E-3</v>
-      </c>
-      <c r="P2">
-        <v>9.4354254989142804E-3</v>
-      </c>
-      <c r="Q2">
-        <v>9.4736842105263164E-3</v>
-      </c>
-      <c r="R2">
-        <v>9.5119429221383524E-3</v>
-      </c>
-      <c r="S2">
-        <v>9.5502016337503867E-3</v>
-      </c>
-      <c r="T2">
-        <v>9.5884603453624245E-3</v>
-      </c>
-      <c r="U2">
-        <v>9.6267190569744605E-3</v>
+      <c r="B2" t="n">
+        <v>0.008899803536345776</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.008938062247957812</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.008976320959569848</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.009014579671181884</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.00905283838279392</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.009091097094405955</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.009129355806017991</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.009167614517630028</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.009205873229242064</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.0092441319408541</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.009282390652466135</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.009320649364078172</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.009358908075690208</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.009397166787302243</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.00943542549891428</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.009473684210526316</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.009511942922138352</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.009550201633750387</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.009588460345362424</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0.00962671905697446</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.45">
-      <c r="A3">
-        <v>0.95499999999999996</v>
-      </c>
-      <c r="B3">
-        <v>8.8998035363457764E-3</v>
-      </c>
-      <c r="C3">
-        <v>8.9380622479578124E-3</v>
-      </c>
-      <c r="D3">
-        <v>8.9763209595698484E-3</v>
-      </c>
-      <c r="E3">
-        <v>9.0145796711818844E-3</v>
-      </c>
-      <c r="F3">
-        <v>9.0528383827939204E-3</v>
-      </c>
-      <c r="G3">
-        <v>9.0910970944059546E-3</v>
-      </c>
-      <c r="H3">
-        <v>9.1293558060179907E-3</v>
-      </c>
-      <c r="I3">
-        <v>9.1676145176300284E-3</v>
-      </c>
-      <c r="J3">
-        <v>9.2058732292420644E-3</v>
-      </c>
-      <c r="K3">
-        <v>9.2441319408541004E-3</v>
-      </c>
-      <c r="L3">
-        <v>9.2823906524661347E-3</v>
-      </c>
-      <c r="M3">
-        <v>9.3206493640781724E-3</v>
-      </c>
-      <c r="N3">
-        <v>9.3589080756902084E-3</v>
-      </c>
-      <c r="O3">
-        <v>9.3971667873022427E-3</v>
-      </c>
-      <c r="P3">
-        <v>9.4354254989142804E-3</v>
-      </c>
-      <c r="Q3">
-        <v>9.4736842105263164E-3</v>
-      </c>
-      <c r="R3">
-        <v>9.5119429221383524E-3</v>
-      </c>
-      <c r="S3">
-        <v>9.5502016337503867E-3</v>
-      </c>
-      <c r="T3">
-        <v>9.5884603453624245E-3</v>
-      </c>
-      <c r="U3">
-        <v>9.6267190569744605E-3</v>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.008899803536345776</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.008938062247957812</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.008976320959569848</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.009014579671181884</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.00905283838279392</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.009091097094405955</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.009129355806017991</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.009167614517630028</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.009205873229242064</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.0092441319408541</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.009282390652466135</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.009320649364078172</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.009358908075690208</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.009397166787302243</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.00943542549891428</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.009473684210526316</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0.009511942922138352</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.009550201633750387</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.009588460345362424</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0.00962671905697446</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixing Flowdata for Veins and Pulm
</commit_message>
<xml_diff>
--- a/BVSimulationFiles/53.xlsx
+++ b/BVSimulationFiles/53.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -483,64 +483,64 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.008899803536345776</v>
+        <v>0.01779960707269155</v>
       </c>
       <c r="C2" t="n">
-        <v>0.008938062247957812</v>
+        <v>0.01787612449591562</v>
       </c>
       <c r="D2" t="n">
-        <v>0.008976320959569848</v>
+        <v>0.0179526419191397</v>
       </c>
       <c r="E2" t="n">
-        <v>0.009014579671181884</v>
+        <v>0.01802915934236377</v>
       </c>
       <c r="F2" t="n">
-        <v>0.00905283838279392</v>
+        <v>0.01810567676558784</v>
       </c>
       <c r="G2" t="n">
-        <v>0.009091097094405955</v>
+        <v>0.01818219418881191</v>
       </c>
       <c r="H2" t="n">
-        <v>0.009129355806017991</v>
+        <v>0.01825871161203598</v>
       </c>
       <c r="I2" t="n">
-        <v>0.009167614517630028</v>
+        <v>0.01833522903526006</v>
       </c>
       <c r="J2" t="n">
-        <v>0.009205873229242064</v>
+        <v>0.01841174645848413</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0092441319408541</v>
+        <v>0.0184882638817082</v>
       </c>
       <c r="L2" t="n">
-        <v>0.009282390652466135</v>
+        <v>0.01856478130493227</v>
       </c>
       <c r="M2" t="n">
-        <v>0.009320649364078172</v>
+        <v>0.01864129872815634</v>
       </c>
       <c r="N2" t="n">
-        <v>0.009358908075690208</v>
+        <v>0.01871781615138042</v>
       </c>
       <c r="O2" t="n">
-        <v>0.009397166787302243</v>
+        <v>0.01879433357460449</v>
       </c>
       <c r="P2" t="n">
-        <v>0.00943542549891428</v>
+        <v>0.01887085099782856</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.009473684210526316</v>
+        <v>0.01894736842105263</v>
       </c>
       <c r="R2" t="n">
-        <v>0.009511942922138352</v>
+        <v>0.0190238858442767</v>
       </c>
       <c r="S2" t="n">
-        <v>0.009550201633750387</v>
+        <v>0.01910040326750077</v>
       </c>
       <c r="T2" t="n">
-        <v>0.009588460345362424</v>
+        <v>0.01917692069072485</v>
       </c>
       <c r="U2" t="n">
-        <v>0.00962671905697446</v>
+        <v>0.01925343811394892</v>
       </c>
     </row>
     <row r="3">
@@ -548,64 +548,64 @@
         <v>0.955</v>
       </c>
       <c r="B3" t="n">
-        <v>0.008899803536345776</v>
+        <v>0.01779960707269155</v>
       </c>
       <c r="C3" t="n">
-        <v>0.008938062247957812</v>
+        <v>0.01787612449591562</v>
       </c>
       <c r="D3" t="n">
-        <v>0.008976320959569848</v>
+        <v>0.0179526419191397</v>
       </c>
       <c r="E3" t="n">
-        <v>0.009014579671181884</v>
+        <v>0.01802915934236377</v>
       </c>
       <c r="F3" t="n">
-        <v>0.00905283838279392</v>
+        <v>0.01810567676558784</v>
       </c>
       <c r="G3" t="n">
-        <v>0.009091097094405955</v>
+        <v>0.01818219418881191</v>
       </c>
       <c r="H3" t="n">
-        <v>0.009129355806017991</v>
+        <v>0.01825871161203598</v>
       </c>
       <c r="I3" t="n">
-        <v>0.009167614517630028</v>
+        <v>0.01833522903526006</v>
       </c>
       <c r="J3" t="n">
-        <v>0.009205873229242064</v>
+        <v>0.01841174645848413</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0092441319408541</v>
+        <v>0.0184882638817082</v>
       </c>
       <c r="L3" t="n">
-        <v>0.009282390652466135</v>
+        <v>0.01856478130493227</v>
       </c>
       <c r="M3" t="n">
-        <v>0.009320649364078172</v>
+        <v>0.01864129872815634</v>
       </c>
       <c r="N3" t="n">
-        <v>0.009358908075690208</v>
+        <v>0.01871781615138042</v>
       </c>
       <c r="O3" t="n">
-        <v>0.009397166787302243</v>
+        <v>0.01879433357460449</v>
       </c>
       <c r="P3" t="n">
-        <v>0.00943542549891428</v>
+        <v>0.01887085099782856</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.009473684210526316</v>
+        <v>0.01894736842105263</v>
       </c>
       <c r="R3" t="n">
-        <v>0.009511942922138352</v>
+        <v>0.0190238858442767</v>
       </c>
       <c r="S3" t="n">
-        <v>0.009550201633750387</v>
+        <v>0.01910040326750077</v>
       </c>
       <c r="T3" t="n">
-        <v>0.009588460345362424</v>
+        <v>0.01917692069072485</v>
       </c>
       <c r="U3" t="n">
-        <v>0.00962671905697446</v>
+        <v>0.01925343811394892</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Resolving Unit Issue for Veinous Flow
</commit_message>
<xml_diff>
--- a/BVSimulationFiles/53.xlsx
+++ b/BVSimulationFiles/53.xlsx
@@ -483,64 +483,64 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01779960707269155</v>
+        <v>0.1779960707269155</v>
       </c>
       <c r="C2" t="n">
-        <v>0.01787612449591562</v>
+        <v>0.1787612449591562</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0179526419191397</v>
+        <v>0.179526419191397</v>
       </c>
       <c r="E2" t="n">
-        <v>0.01802915934236377</v>
+        <v>0.1802915934236377</v>
       </c>
       <c r="F2" t="n">
-        <v>0.01810567676558784</v>
+        <v>0.1810567676558784</v>
       </c>
       <c r="G2" t="n">
-        <v>0.01818219418881191</v>
+        <v>0.1818219418881191</v>
       </c>
       <c r="H2" t="n">
-        <v>0.01825871161203598</v>
+        <v>0.1825871161203598</v>
       </c>
       <c r="I2" t="n">
-        <v>0.01833522903526006</v>
+        <v>0.1833522903526006</v>
       </c>
       <c r="J2" t="n">
-        <v>0.01841174645848413</v>
+        <v>0.1841174645848413</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0184882638817082</v>
+        <v>0.184882638817082</v>
       </c>
       <c r="L2" t="n">
-        <v>0.01856478130493227</v>
+        <v>0.1856478130493227</v>
       </c>
       <c r="M2" t="n">
-        <v>0.01864129872815634</v>
+        <v>0.1864129872815634</v>
       </c>
       <c r="N2" t="n">
-        <v>0.01871781615138042</v>
+        <v>0.1871781615138042</v>
       </c>
       <c r="O2" t="n">
-        <v>0.01879433357460449</v>
+        <v>0.1879433357460449</v>
       </c>
       <c r="P2" t="n">
-        <v>0.01887085099782856</v>
+        <v>0.1887085099782856</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.01894736842105263</v>
+        <v>0.1894736842105263</v>
       </c>
       <c r="R2" t="n">
-        <v>0.0190238858442767</v>
+        <v>0.190238858442767</v>
       </c>
       <c r="S2" t="n">
-        <v>0.01910040326750077</v>
+        <v>0.1910040326750077</v>
       </c>
       <c r="T2" t="n">
-        <v>0.01917692069072485</v>
+        <v>0.1917692069072485</v>
       </c>
       <c r="U2" t="n">
-        <v>0.01925343811394892</v>
+        <v>0.1925343811394892</v>
       </c>
     </row>
     <row r="3">
@@ -548,64 +548,64 @@
         <v>0.955</v>
       </c>
       <c r="B3" t="n">
-        <v>0.01779960707269155</v>
+        <v>0.1779960707269155</v>
       </c>
       <c r="C3" t="n">
-        <v>0.01787612449591562</v>
+        <v>0.1787612449591562</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0179526419191397</v>
+        <v>0.179526419191397</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01802915934236377</v>
+        <v>0.1802915934236377</v>
       </c>
       <c r="F3" t="n">
-        <v>0.01810567676558784</v>
+        <v>0.1810567676558784</v>
       </c>
       <c r="G3" t="n">
-        <v>0.01818219418881191</v>
+        <v>0.1818219418881191</v>
       </c>
       <c r="H3" t="n">
-        <v>0.01825871161203598</v>
+        <v>0.1825871161203598</v>
       </c>
       <c r="I3" t="n">
-        <v>0.01833522903526006</v>
+        <v>0.1833522903526006</v>
       </c>
       <c r="J3" t="n">
-        <v>0.01841174645848413</v>
+        <v>0.1841174645848413</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0184882638817082</v>
+        <v>0.184882638817082</v>
       </c>
       <c r="L3" t="n">
-        <v>0.01856478130493227</v>
+        <v>0.1856478130493227</v>
       </c>
       <c r="M3" t="n">
-        <v>0.01864129872815634</v>
+        <v>0.1864129872815634</v>
       </c>
       <c r="N3" t="n">
-        <v>0.01871781615138042</v>
+        <v>0.1871781615138042</v>
       </c>
       <c r="O3" t="n">
-        <v>0.01879433357460449</v>
+        <v>0.1879433357460449</v>
       </c>
       <c r="P3" t="n">
-        <v>0.01887085099782856</v>
+        <v>0.1887085099782856</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.01894736842105263</v>
+        <v>0.1894736842105263</v>
       </c>
       <c r="R3" t="n">
-        <v>0.0190238858442767</v>
+        <v>0.190238858442767</v>
       </c>
       <c r="S3" t="n">
-        <v>0.01910040326750077</v>
+        <v>0.1910040326750077</v>
       </c>
       <c r="T3" t="n">
-        <v>0.01917692069072485</v>
+        <v>0.1917692069072485</v>
       </c>
       <c r="U3" t="n">
-        <v>0.01925343811394892</v>
+        <v>0.1925343811394892</v>
       </c>
     </row>
   </sheetData>

</xml_diff>